<commit_message>
docs: prepare phase two release acceptance
</commit_message>
<xml_diff>
--- a/docs/第二阶段人工测试表.xlsx
+++ b/docs/第二阶段人工测试表.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模块覆盖" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'测试用例'!$A$1:$Q$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'测试用例'!$A$1:$Q$63</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -608,7 +608,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>0.2.0</t>
+          <t>0.3.0</t>
         </is>
       </c>
       <c r="C4" s="4" t="n"/>
@@ -696,6 +696,13 @@
           <t>填写约定</t>
         </is>
       </c>
+      <c r="B10" s="4" t="n"/>
+      <c r="C10" s="4" t="n"/>
+      <c r="D10" s="4" t="n"/>
+      <c r="E10" s="4" t="n"/>
+      <c r="F10" s="4" t="n"/>
+      <c r="G10" s="4" t="n"/>
+      <c r="H10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -775,6 +782,13 @@
           <t>当前实现注意事项</t>
         </is>
       </c>
+      <c r="B16" s="4" t="n"/>
+      <c r="C16" s="4" t="n"/>
+      <c r="D16" s="4" t="n"/>
+      <c r="E16" s="4" t="n"/>
+      <c r="F16" s="4" t="n"/>
+      <c r="G16" s="4" t="n"/>
+      <c r="H16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -782,6 +796,13 @@
           <t>1. 收集箱视图默认只显示 status=pending 且未删除的条目。</t>
         </is>
       </c>
+      <c r="B17" s="4" t="n"/>
+      <c r="C17" s="4" t="n"/>
+      <c r="D17" s="4" t="n"/>
+      <c r="E17" s="4" t="n"/>
+      <c r="F17" s="4" t="n"/>
+      <c r="G17" s="4" t="n"/>
+      <c r="H17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -789,13 +810,27 @@
           <t>2. 主窗口和快速记录窗口的关闭动作都会隐藏窗口，不直接退出应用。</t>
         </is>
       </c>
+      <c r="B18" s="4" t="n"/>
+      <c r="C18" s="4" t="n"/>
+      <c r="D18" s="4" t="n"/>
+      <c r="E18" s="4" t="n"/>
+      <c r="F18" s="4" t="n"/>
+      <c r="G18" s="4" t="n"/>
+      <c r="H18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>3. Markdown 导出覆盖全部未永久删除条目，包括回收站中的条目。</t>
-        </is>
-      </c>
+          <t>3. Markdown 导出只包含未进入回收站的条目。</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n"/>
+      <c r="C19" s="4" t="n"/>
+      <c r="D19" s="4" t="n"/>
+      <c r="E19" s="4" t="n"/>
+      <c r="F19" s="4" t="n"/>
+      <c r="G19" s="4" t="n"/>
+      <c r="H19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -803,6 +838,13 @@
           <t>4. 全局快捷键、托盘、开机自启动、打开目录按钮都必须在真实 Windows 桌面会话中验证。</t>
         </is>
       </c>
+      <c r="B20" s="4" t="n"/>
+      <c r="C20" s="4" t="n"/>
+      <c r="D20" s="4" t="n"/>
+      <c r="E20" s="4" t="n"/>
+      <c r="F20" s="4" t="n"/>
+      <c r="G20" s="4" t="n"/>
+      <c r="H20" s="5" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -810,6 +852,13 @@
           <t>5. 搜索当前已覆盖标题、当前内容、原始内容和标签名四类命中路径。</t>
         </is>
       </c>
+      <c r="B21" s="4" t="n"/>
+      <c r="C21" s="4" t="n"/>
+      <c r="D21" s="4" t="n"/>
+      <c r="E21" s="4" t="n"/>
+      <c r="F21" s="4" t="n"/>
+      <c r="G21" s="4" t="n"/>
+      <c r="H21" s="5" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="18">
@@ -842,7 +891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q46"/>
+  <dimension ref="A1:Q63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3536,7 +3585,7 @@
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>导出覆盖全部未永久删除条目</t>
+          <t>导出覆盖全部未进入回收站条目</t>
         </is>
       </c>
       <c r="E39" s="10" t="inlineStr">
@@ -3573,8 +3622,8 @@
       </c>
       <c r="K39" s="9" t="inlineStr">
         <is>
-          <t>1. 导出数量与当前未永久删除条目总数一致
-2. 回收站中的条目也会被导出
+          <t>1. 导出数量与所有未进入回收站条目数一致
+2. 回收站条目不导出，恢复后可再次导出
 3. 无文件被覆盖报错</t>
         </is>
       </c>
@@ -4080,8 +4129,1170 @@
       <c r="P46" s="10" t="inlineStr"/>
       <c r="Q46" s="9" t="inlineStr"/>
     </row>
+    <row r="47">
+      <c r="A47" s="9" t="inlineStr">
+        <is>
+          <t>KB-01</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>知识节点</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>沉淀</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>条目沉淀为知识且从收集箱移除</t>
+        </is>
+      </c>
+      <c r="E47" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F47" s="10" t="inlineStr">
+        <is>
+          <t>必回归</t>
+        </is>
+      </c>
+      <c r="G47" s="10" t="inlineStr">
+        <is>
+          <t>已自动覆盖</t>
+        </is>
+      </c>
+      <c r="H47" s="9" t="inlineStr">
+        <is>
+          <t>桌面交互</t>
+        </is>
+      </c>
+      <c r="I47" s="9" t="inlineStr">
+        <is>
+          <t>收集箱有一条已保存且标题非空的捕获条目</t>
+        </is>
+      </c>
+      <c r="J47" s="9" t="inlineStr">
+        <is>
+          <t>1. 打开条目
+2. 点击“沉淀”
+3. 切换收集箱和知识库</t>
+        </is>
+      </c>
+      <c r="K47" s="9" t="inlineStr">
+        <is>
+          <t>条目 ID、正文、原文和标签不变；从收集箱移除并出现在知识库</t>
+        </is>
+      </c>
+      <c r="L47" s="9" t="n"/>
+      <c r="M47" s="10" t="inlineStr">
+        <is>
+          <t>未执行</t>
+        </is>
+      </c>
+      <c r="N47" s="10" t="n"/>
+      <c r="O47" s="10" t="n"/>
+      <c r="P47" s="10" t="n"/>
+      <c r="Q47" s="9" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>KB-02</t>
+        </is>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>知识节点</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>标题唯一性</t>
+        </is>
+      </c>
+      <c r="D48" s="9" t="inlineStr">
+        <is>
+          <t>重复规范化标题被拒绝且正文不丢</t>
+        </is>
+      </c>
+      <c r="E48" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F48" s="10" t="inlineStr">
+        <is>
+          <t>必回归</t>
+        </is>
+      </c>
+      <c r="G48" s="10" t="inlineStr">
+        <is>
+          <t>已自动覆盖</t>
+        </is>
+      </c>
+      <c r="H48" s="9" t="inlineStr">
+        <is>
+          <t>桌面交互</t>
+        </is>
+      </c>
+      <c r="I48" s="9" t="inlineStr">
+        <is>
+          <t>已有知识标题“Same Title”；另一条捕获条目标题为“same   title”</t>
+        </is>
+      </c>
+      <c r="J48" s="9" t="inlineStr">
+        <is>
+          <t>1. 尝试沉淀第二条
+2. 观察错误
+3. 重新打开条目</t>
+        </is>
+      </c>
+      <c r="K48" s="9" t="inlineStr">
+        <is>
+          <t>显示标题冲突；第二条的正文、标题和 revision 不变</t>
+        </is>
+      </c>
+      <c r="L48" s="9" t="n"/>
+      <c r="M48" s="10" t="inlineStr">
+        <is>
+          <t>未执行</t>
+        </is>
+      </c>
+      <c r="N48" s="10" t="n"/>
+      <c r="O48" s="10" t="n"/>
+      <c r="P48" s="10" t="n"/>
+      <c r="Q48" s="9" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="9" t="inlineStr">
+        <is>
+          <t>KB-03</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>知识节点</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="inlineStr">
+        <is>
+          <t>移出</t>
+        </is>
+      </c>
+      <c r="D49" s="9" t="inlineStr">
+        <is>
+          <t>移出知识库后回到捕获态</t>
+        </is>
+      </c>
+      <c r="E49" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F49" s="10" t="inlineStr">
+        <is>
+          <t>建议回归</t>
+        </is>
+      </c>
+      <c r="G49" s="10" t="inlineStr">
+        <is>
+          <t>已自动覆盖</t>
+        </is>
+      </c>
+      <c r="H49" s="9" t="inlineStr">
+        <is>
+          <t>桌面交互</t>
+        </is>
+      </c>
+      <c r="I49" s="9" t="inlineStr">
+        <is>
+          <t>知识库中有一条知识节点</t>
+        </is>
+      </c>
+      <c r="J49" s="9" t="inlineStr">
+        <is>
+          <t>1. 打开节点
+2. 点击“移出知识库”
+3. 查看知识库与收集箱</t>
+        </is>
+      </c>
+      <c r="K49" s="9" t="inlineStr">
+        <is>
+          <t>知识状态清除，节点从知识库消失；待处理条目回到收集箱</t>
+        </is>
+      </c>
+      <c r="L49" s="9" t="n"/>
+      <c r="M49" s="10" t="inlineStr">
+        <is>
+          <t>未执行</t>
+        </is>
+      </c>
+      <c r="N49" s="10" t="n"/>
+      <c r="O49" s="10" t="n"/>
+      <c r="P49" s="10" t="n"/>
+      <c r="Q49" s="9" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>KB-04</t>
+        </is>
+      </c>
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>知识节点</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>历史标题</t>
+        </is>
+      </c>
+      <c r="D50" s="9" t="inlineStr">
+        <is>
+          <t>重命名后旧标题链接继续解析</t>
+        </is>
+      </c>
+      <c r="E50" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F50" s="10" t="inlineStr">
+        <is>
+          <t>必回归</t>
+        </is>
+      </c>
+      <c r="G50" s="10" t="inlineStr">
+        <is>
+          <t>已自动覆盖</t>
+        </is>
+      </c>
+      <c r="H50" s="9" t="inlineStr">
+        <is>
+          <t>桌面交互</t>
+        </is>
+      </c>
+      <c r="I50" s="9" t="inlineStr">
+        <is>
+          <t>来源条目正文含 [[旧标题]]；目标为知识节点</t>
+        </is>
+      </c>
+      <c r="J50" s="9" t="inlineStr">
+        <is>
+          <t>1. 将目标重命名为新标题
+2. 查看目标反链和来源出链</t>
+        </is>
+      </c>
+      <c r="K50" s="9" t="inlineStr">
+        <is>
+          <t>[[旧标题]] 仍指向同一 ID；历史标题可见，正文不被改写</t>
+        </is>
+      </c>
+      <c r="L50" s="9" t="n"/>
+      <c r="M50" s="10" t="inlineStr">
+        <is>
+          <t>未执行</t>
+        </is>
+      </c>
+      <c r="N50" s="10" t="n"/>
+      <c r="O50" s="10" t="n"/>
+      <c r="P50" s="10" t="n"/>
+      <c r="Q50" s="9" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t>LK-01</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>知识关联</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="inlineStr">
+        <is>
+          <t>WikiLink 补全</t>
+        </is>
+      </c>
+      <c r="D51" s="9" t="inlineStr">
+        <is>
+          <t>[[ 补全插入 canonical title</t>
+        </is>
+      </c>
+      <c r="E51" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F51" s="10" t="inlineStr">
+        <is>
+          <t>必回归</t>
+        </is>
+      </c>
+      <c r="G51" s="10" t="inlineStr">
+        <is>
+          <t>已自动覆盖</t>
+        </is>
+      </c>
+      <c r="H51" s="9" t="inlineStr">
+        <is>
+          <t>桌面交互</t>
+        </is>
+      </c>
+      <c r="I51" s="9" t="inlineStr">
+        <is>
+          <t>库中已有知识节点“知识库”</t>
+        </is>
+      </c>
+      <c r="J51" s="9" t="inlineStr">
+        <is>
+          <t>1. 在正文输入 [[知
+2. 用键盘选择建议
+3. 继续输入并等待保存</t>
+        </is>
+      </c>
+      <c r="K51" s="9" t="inlineStr">
+        <is>
+          <t>插入 [[知识库]]，光标位于闭括号后，正文自动保存</t>
+        </is>
+      </c>
+      <c r="L51" s="9" t="n"/>
+      <c r="M51" s="10" t="inlineStr">
+        <is>
+          <t>未执行</t>
+        </is>
+      </c>
+      <c r="N51" s="10" t="n"/>
+      <c r="O51" s="10" t="n"/>
+      <c r="P51" s="10" t="n"/>
+      <c r="Q51" s="9" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="9" t="inlineStr">
+        <is>
+          <t>LK-02</t>
+        </is>
+      </c>
+      <c r="B52" s="9" t="inlineStr">
+        <is>
+          <t>知识关联</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="inlineStr">
+        <is>
+          <t>关系面板</t>
+        </is>
+      </c>
+      <c r="D52" s="9" t="inlineStr">
+        <is>
+          <t>出链与反链 occurrence 正确</t>
+        </is>
+      </c>
+      <c r="E52" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F52" s="10" t="inlineStr">
+        <is>
+          <t>必回归</t>
+        </is>
+      </c>
+      <c r="G52" s="10" t="inlineStr">
+        <is>
+          <t>已自动覆盖</t>
+        </is>
+      </c>
+      <c r="H52" s="9" t="inlineStr">
+        <is>
+          <t>桌面交互</t>
+        </is>
+      </c>
+      <c r="I52" s="9" t="inlineStr">
+        <is>
+          <t>来源正文两次引用同一知识节点</t>
+        </is>
+      </c>
+      <c r="J52" s="9" t="inlineStr">
+        <is>
+          <t>1. 打开来源和目标
+2. 查看出链、反向链接及次数</t>
+        </is>
+      </c>
+      <c r="K52" s="9" t="inlineStr">
+        <is>
+          <t>来源只列一个出链且次数为 2；目标只列一个反链且次数为 2</t>
+        </is>
+      </c>
+      <c r="L52" s="9" t="n"/>
+      <c r="M52" s="10" t="inlineStr">
+        <is>
+          <t>未执行</t>
+        </is>
+      </c>
+      <c r="N52" s="10" t="n"/>
+      <c r="O52" s="10" t="n"/>
+      <c r="P52" s="10" t="n"/>
+      <c r="Q52" s="9" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="9" t="inlineStr">
+        <is>
+          <t>LK-03</t>
+        </is>
+      </c>
+      <c r="B53" s="9" t="inlineStr">
+        <is>
+          <t>知识关联</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="inlineStr">
+        <is>
+          <t>未解析</t>
+        </is>
+      </c>
+      <c r="D53" s="9" t="inlineStr">
+        <is>
+          <t>未解析链接可见</t>
+        </is>
+      </c>
+      <c r="E53" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F53" s="10" t="inlineStr">
+        <is>
+          <t>建议回归</t>
+        </is>
+      </c>
+      <c r="G53" s="10" t="inlineStr">
+        <is>
+          <t>已自动覆盖</t>
+        </is>
+      </c>
+      <c r="H53" s="9" t="inlineStr">
+        <is>
+          <t>桌面交互</t>
+        </is>
+      </c>
+      <c r="I53" s="9" t="inlineStr">
+        <is>
+          <t>正文含 [[不存在的标题]]</t>
+        </is>
+      </c>
+      <c r="J53" s="9" t="inlineStr">
+        <is>
+          <t>1. 保存正文
+2. 查看关系面板</t>
+        </is>
+      </c>
+      <c r="K53" s="9" t="inlineStr">
+        <is>
+          <t>未解析区显示原始标题及 occurrence，不伪装成空关系</t>
+        </is>
+      </c>
+      <c r="L53" s="9" t="n"/>
+      <c r="M53" s="10" t="inlineStr">
+        <is>
+          <t>未执行</t>
+        </is>
+      </c>
+      <c r="N53" s="10" t="n"/>
+      <c r="O53" s="10" t="n"/>
+      <c r="P53" s="10" t="n"/>
+      <c r="Q53" s="9" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="9" t="inlineStr">
+        <is>
+          <t>LK-04</t>
+        </is>
+      </c>
+      <c r="B54" s="9" t="inlineStr">
+        <is>
+          <t>知识关联</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>跨窗口刷新</t>
+        </is>
+      </c>
+      <c r="D54" s="9" t="inlineStr">
+        <is>
+          <t>快速记录新增反链后主窗口刷新</t>
+        </is>
+      </c>
+      <c r="E54" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F54" s="10" t="inlineStr">
+        <is>
+          <t>必回归</t>
+        </is>
+      </c>
+      <c r="G54" s="10" t="inlineStr">
+        <is>
+          <t>部分自动覆盖</t>
+        </is>
+      </c>
+      <c r="H54" s="9" t="inlineStr">
+        <is>
+          <t>系统集成</t>
+        </is>
+      </c>
+      <c r="I54" s="9" t="inlineStr">
+        <is>
+          <t>主窗口正打开某知识节点</t>
+        </is>
+      </c>
+      <c r="J54" s="9" t="inlineStr">
+        <is>
+          <t>1. 用快速记录提交包含该节点 WikiLink 的新条目
+2. 观察主窗口反链</t>
+        </is>
+      </c>
+      <c r="K54" s="9" t="inlineStr">
+        <is>
+          <t>未覆盖本地未保存编辑；刷新列表、标签和反链，新来源可见</t>
+        </is>
+      </c>
+      <c r="L54" s="9" t="n"/>
+      <c r="M54" s="10" t="inlineStr">
+        <is>
+          <t>未执行</t>
+        </is>
+      </c>
+      <c r="N54" s="10" t="n"/>
+      <c r="O54" s="10" t="n"/>
+      <c r="P54" s="10" t="n"/>
+      <c r="Q54" s="9" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="9" t="inlineStr">
+        <is>
+          <t>LK-05</t>
+        </is>
+      </c>
+      <c r="B55" s="9" t="inlineStr">
+        <is>
+          <t>知识关联</t>
+        </is>
+      </c>
+      <c r="C55" s="9" t="inlineStr">
+        <is>
+          <t>回收站</t>
+        </is>
+      </c>
+      <c r="D55" s="9" t="inlineStr">
+        <is>
+          <t>目标移入回收站和恢复不丢关系</t>
+        </is>
+      </c>
+      <c r="E55" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F55" s="10" t="inlineStr">
+        <is>
+          <t>建议回归</t>
+        </is>
+      </c>
+      <c r="G55" s="10" t="inlineStr">
+        <is>
+          <t>已自动覆盖</t>
+        </is>
+      </c>
+      <c r="H55" s="9" t="inlineStr">
+        <is>
+          <t>桌面交互</t>
+        </is>
+      </c>
+      <c r="I55" s="9" t="inlineStr">
+        <is>
+          <t>已有指向知识节点的出链</t>
+        </is>
+      </c>
+      <c r="J55" s="9" t="inlineStr">
+        <is>
+          <t>1. 将目标移入回收站
+2. 查看来源关系
+3. 恢复目标</t>
+        </is>
+      </c>
+      <c r="K55" s="9" t="inlineStr">
+        <is>
+          <t>关系持续保留并显示回收站标记；恢复后立即正常</t>
+        </is>
+      </c>
+      <c r="L55" s="9" t="n"/>
+      <c r="M55" s="10" t="inlineStr">
+        <is>
+          <t>未执行</t>
+        </is>
+      </c>
+      <c r="N55" s="10" t="n"/>
+      <c r="O55" s="10" t="n"/>
+      <c r="P55" s="10" t="n"/>
+      <c r="Q55" s="9" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="9" t="inlineStr">
+        <is>
+          <t>LK-06</t>
+        </is>
+      </c>
+      <c r="B56" s="9" t="inlineStr">
+        <is>
+          <t>知识关联</t>
+        </is>
+      </c>
+      <c r="C56" s="9" t="inlineStr">
+        <is>
+          <t>永久删除</t>
+        </is>
+      </c>
+      <c r="D56" s="9" t="inlineStr">
+        <is>
+          <t>永久删除目标后文本保留且关系变未解析</t>
+        </is>
+      </c>
+      <c r="E56" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F56" s="10" t="inlineStr">
+        <is>
+          <t>建议回归</t>
+        </is>
+      </c>
+      <c r="G56" s="10" t="inlineStr">
+        <is>
+          <t>已自动覆盖</t>
+        </is>
+      </c>
+      <c r="H56" s="9" t="inlineStr">
+        <is>
+          <t>桌面交互</t>
+        </is>
+      </c>
+      <c r="I56" s="9" t="inlineStr">
+        <is>
+          <t>回收站中有被其他条目引用的知识节点</t>
+        </is>
+      </c>
+      <c r="J56" s="9" t="inlineStr">
+        <is>
+          <t>1. 永久删除目标
+2. 打开来源条目</t>
+        </is>
+      </c>
+      <c r="K56" s="9" t="inlineStr">
+        <is>
+          <t>来源正文中 WikiLink 文本不变；已解析关系变为未解析</t>
+        </is>
+      </c>
+      <c r="L56" s="9" t="n"/>
+      <c r="M56" s="10" t="inlineStr">
+        <is>
+          <t>未执行</t>
+        </is>
+      </c>
+      <c r="N56" s="10" t="n"/>
+      <c r="O56" s="10" t="n"/>
+      <c r="P56" s="10" t="n"/>
+      <c r="Q56" s="9" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="9" t="inlineStr">
+        <is>
+          <t>SR-01</t>
+        </is>
+      </c>
+      <c r="B57" s="9" t="inlineStr">
+        <is>
+          <t>增强搜索</t>
+        </is>
+      </c>
+      <c r="C57" s="9" t="inlineStr">
+        <is>
+          <t>trigram</t>
+        </is>
+      </c>
+      <c r="D57" s="9" t="inlineStr">
+        <is>
+          <t>三字中文子串搜索命中</t>
+        </is>
+      </c>
+      <c r="E57" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F57" s="10" t="inlineStr">
+        <is>
+          <t>必回归</t>
+        </is>
+      </c>
+      <c r="G57" s="10" t="inlineStr">
+        <is>
+          <t>已自动覆盖</t>
+        </is>
+      </c>
+      <c r="H57" s="9" t="inlineStr">
+        <is>
+          <t>桌面交互</t>
+        </is>
+      </c>
+      <c r="I57" s="9" t="inlineStr">
+        <is>
+          <t>条目正文含“第二阶段知识库全文搜索”</t>
+        </is>
+      </c>
+      <c r="J57" s="9" t="inlineStr">
+        <is>
+          <t>1. 搜索“知识库”
+2. 观察结果</t>
+        </is>
+      </c>
+      <c r="K57" s="9" t="inlineStr">
+        <is>
+          <t>命中目标条目，走 trigram FTS 而不是 %LIKE% 全表扫描</t>
+        </is>
+      </c>
+      <c r="L57" s="9" t="n"/>
+      <c r="M57" s="10" t="inlineStr">
+        <is>
+          <t>未执行</t>
+        </is>
+      </c>
+      <c r="N57" s="10" t="n"/>
+      <c r="O57" s="10" t="n"/>
+      <c r="P57" s="10" t="n"/>
+      <c r="Q57" s="9" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="9" t="inlineStr">
+        <is>
+          <t>SR-02</t>
+        </is>
+      </c>
+      <c r="B58" s="9" t="inlineStr">
+        <is>
+          <t>增强搜索</t>
+        </is>
+      </c>
+      <c r="C58" s="9" t="inlineStr">
+        <is>
+          <t>排名与片段</t>
+        </is>
+      </c>
+      <c r="D58" s="9" t="inlineStr">
+        <is>
+          <t>搜索相关度和命中片段正确</t>
+        </is>
+      </c>
+      <c r="E58" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F58" s="10" t="inlineStr">
+        <is>
+          <t>建议回归</t>
+        </is>
+      </c>
+      <c r="G58" s="10" t="inlineStr">
+        <is>
+          <t>已自动覆盖</t>
+        </is>
+      </c>
+      <c r="H58" s="9" t="inlineStr">
+        <is>
+          <t>桌面交互</t>
+        </is>
+      </c>
+      <c r="I58" s="9" t="inlineStr">
+        <is>
+          <t>准备标题、正文、标签和历史标题中不同强度的命中</t>
+        </is>
+      </c>
+      <c r="J58" s="9" t="inlineStr">
+        <is>
+          <t>1. 输入三字以上关键词
+2. 查看排序和高亮片段</t>
+        </is>
+      </c>
+      <c r="K58" s="9" t="inlineStr">
+        <is>
+          <t>标题等高权重命中优先；片段文字正确且高亮不执行 HTML</t>
+        </is>
+      </c>
+      <c r="L58" s="9" t="n"/>
+      <c r="M58" s="10" t="inlineStr">
+        <is>
+          <t>未执行</t>
+        </is>
+      </c>
+      <c r="N58" s="10" t="n"/>
+      <c r="O58" s="10" t="n"/>
+      <c r="P58" s="10" t="n"/>
+      <c r="Q58" s="9" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="9" t="inlineStr">
+        <is>
+          <t>SR-03</t>
+        </is>
+      </c>
+      <c r="B59" s="9" t="inlineStr">
+        <is>
+          <t>增强搜索</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="inlineStr">
+        <is>
+          <t>短查询回退</t>
+        </is>
+      </c>
+      <c r="D59" s="9" t="inlineStr">
+        <is>
+          <t>两字查询 LIKE 回退</t>
+        </is>
+      </c>
+      <c r="E59" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F59" s="10" t="inlineStr">
+        <is>
+          <t>必回归</t>
+        </is>
+      </c>
+      <c r="G59" s="10" t="inlineStr">
+        <is>
+          <t>已自动覆盖</t>
+        </is>
+      </c>
+      <c r="H59" s="9" t="inlineStr">
+        <is>
+          <t>桌面交互</t>
+        </is>
+      </c>
+      <c r="I59" s="9" t="inlineStr">
+        <is>
+          <t>条目标题、正文或历史标题含“知识”</t>
+        </is>
+      </c>
+      <c r="J59" s="9" t="inlineStr">
+        <is>
+          <t>1. 搜索“知识”
+2. 观察结果</t>
+        </is>
+      </c>
+      <c r="K59" s="9" t="inlineStr">
+        <is>
+          <t>两字查询通过按词 LIKE 正确命中，不因 trigram 索引返回假空</t>
+        </is>
+      </c>
+      <c r="L59" s="9" t="n"/>
+      <c r="M59" s="10" t="inlineStr">
+        <is>
+          <t>未执行</t>
+        </is>
+      </c>
+      <c r="N59" s="10" t="n"/>
+      <c r="O59" s="10" t="n"/>
+      <c r="P59" s="10" t="n"/>
+      <c r="Q59" s="9" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="9" t="inlineStr">
+        <is>
+          <t>SR-04</t>
+        </is>
+      </c>
+      <c r="B60" s="9" t="inlineStr">
+        <is>
+          <t>增强搜索</t>
+        </is>
+      </c>
+      <c r="C60" s="9" t="inlineStr">
+        <is>
+          <t>视图筛选</t>
+        </is>
+      </c>
+      <c r="D60" s="9" t="inlineStr">
+        <is>
+          <t>知识库视图与搜索筛选互不污染</t>
+        </is>
+      </c>
+      <c r="E60" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F60" s="10" t="inlineStr">
+        <is>
+          <t>建议回归</t>
+        </is>
+      </c>
+      <c r="G60" s="10" t="inlineStr">
+        <is>
+          <t>部分自动覆盖</t>
+        </is>
+      </c>
+      <c r="H60" s="9" t="inlineStr">
+        <is>
+          <t>桌面交互</t>
+        </is>
+      </c>
+      <c r="I60" s="9" t="inlineStr">
+        <is>
+          <t>同时存在捕获态和知识态条目</t>
+        </is>
+      </c>
+      <c r="J60" s="9" t="inlineStr">
+        <is>
+          <t>1. 在知识库搜索并切换类型/状态
+2. 切换搜索、收集箱后返回</t>
+        </is>
+      </c>
+      <c r="K60" s="9" t="inlineStr">
+        <is>
+          <t>各视图使用自身 knowledge state 语义，切换后不残留错误筛选</t>
+        </is>
+      </c>
+      <c r="L60" s="9" t="n"/>
+      <c r="M60" s="10" t="inlineStr">
+        <is>
+          <t>未执行</t>
+        </is>
+      </c>
+      <c r="N60" s="10" t="n"/>
+      <c r="O60" s="10" t="n"/>
+      <c r="P60" s="10" t="n"/>
+      <c r="Q60" s="9" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="9" t="inlineStr">
+        <is>
+          <t>IX-01</t>
+        </is>
+      </c>
+      <c r="B61" s="9" t="inlineStr">
+        <is>
+          <t>索引维护</t>
+        </is>
+      </c>
+      <c r="C61" s="9" t="inlineStr">
+        <is>
+          <t>重建</t>
+        </is>
+      </c>
+      <c r="D61" s="9" t="inlineStr">
+        <is>
+          <t>重建索引不修改正文和 revision</t>
+        </is>
+      </c>
+      <c r="E61" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F61" s="10" t="inlineStr">
+        <is>
+          <t>必回归</t>
+        </is>
+      </c>
+      <c r="G61" s="10" t="inlineStr">
+        <is>
+          <t>已自动覆盖</t>
+        </is>
+      </c>
+      <c r="H61" s="9" t="inlineStr">
+        <is>
+          <t>桌面交互+数据校验</t>
+        </is>
+      </c>
+      <c r="I61" s="9" t="inlineStr">
+        <is>
+          <t>库中有知识节点、WikiLink 和未解析链接</t>
+        </is>
+      </c>
+      <c r="J61" s="9" t="inlineStr">
+        <is>
+          <t>1. 记录正文、原文和 revision
+2. 设置页点击重建索引
+3. 再次核对</t>
+        </is>
+      </c>
+      <c r="K61" s="9" t="inlineStr">
+        <is>
+          <t>重建成功并显示统计；正文、原文、revision 完全不变</t>
+        </is>
+      </c>
+      <c r="L61" s="9" t="n"/>
+      <c r="M61" s="10" t="inlineStr">
+        <is>
+          <t>未执行</t>
+        </is>
+      </c>
+      <c r="N61" s="10" t="n"/>
+      <c r="O61" s="10" t="n"/>
+      <c r="P61" s="10" t="n"/>
+      <c r="Q61" s="9" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="9" t="inlineStr">
+        <is>
+          <t>EX-04</t>
+        </is>
+      </c>
+      <c r="B62" s="9" t="inlineStr">
+        <is>
+          <t>设置与导出</t>
+        </is>
+      </c>
+      <c r="C62" s="9" t="inlineStr">
+        <is>
+          <t>Markdown 导出</t>
+        </is>
+      </c>
+      <c r="D62" s="9" t="inlineStr">
+        <is>
+          <t>导出包含知识状态、沉淀时间和 aliases</t>
+        </is>
+      </c>
+      <c r="E62" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F62" s="10" t="inlineStr">
+        <is>
+          <t>建议回归</t>
+        </is>
+      </c>
+      <c r="G62" s="10" t="inlineStr">
+        <is>
+          <t>已自动覆盖</t>
+        </is>
+      </c>
+      <c r="H62" s="9" t="inlineStr">
+        <is>
+          <t>文件校验</t>
+        </is>
+      </c>
+      <c r="I62" s="9" t="inlineStr">
+        <is>
+          <t>知识节点已重命名且正文含 WikiLink</t>
+        </is>
+      </c>
+      <c r="J62" s="9" t="inlineStr">
+        <is>
+          <t>1. 导出 Markdown
+2. 解析 frontmatter 与正文</t>
+        </is>
+      </c>
+      <c r="K62" s="9" t="inlineStr">
+        <is>
+          <t>frontmatter 包含 knowledge_state、knowledge_promoted_at、aliases；WikiLink 文本原样保留</t>
+        </is>
+      </c>
+      <c r="L62" s="9" t="n"/>
+      <c r="M62" s="10" t="inlineStr">
+        <is>
+          <t>未执行</t>
+        </is>
+      </c>
+      <c r="N62" s="10" t="n"/>
+      <c r="O62" s="10" t="n"/>
+      <c r="P62" s="10" t="n"/>
+      <c r="Q62" s="9" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="9" t="inlineStr">
+        <is>
+          <t>DS-06</t>
+        </is>
+      </c>
+      <c r="B63" s="9" t="inlineStr">
+        <is>
+          <t>桌面集成与持久化</t>
+        </is>
+      </c>
+      <c r="C63" s="9" t="inlineStr">
+        <is>
+          <t>备份恢复</t>
+        </is>
+      </c>
+      <c r="D63" s="9" t="inlineStr">
+        <is>
+          <t>备份恢复知识状态、别名和反链</t>
+        </is>
+      </c>
+      <c r="E63" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F63" s="10" t="inlineStr">
+        <is>
+          <t>必回归</t>
+        </is>
+      </c>
+      <c r="G63" s="10" t="inlineStr">
+        <is>
+          <t>已自动覆盖</t>
+        </is>
+      </c>
+      <c r="H63" s="9" t="inlineStr">
+        <is>
+          <t>系统集成+数据校验</t>
+        </is>
+      </c>
+      <c r="I63" s="9" t="inlineStr">
+        <is>
+          <t>库中存在知识节点、历史标题、反链和备份</t>
+        </is>
+      </c>
+      <c r="J63" s="9" t="inlineStr">
+        <is>
+          <t>1. 恢复备份
+2. 检查知识库、搜索和关系面板</t>
+        </is>
+      </c>
+      <c r="K63" s="9" t="inlineStr">
+        <is>
+          <t>知识状态和 aliases 恢复；反链 occurrence 按正文重建；旧标题可搜索</t>
+        </is>
+      </c>
+      <c r="L63" s="9" t="n"/>
+      <c r="M63" s="10" t="inlineStr">
+        <is>
+          <t>未执行</t>
+        </is>
+      </c>
+      <c r="N63" s="10" t="n"/>
+      <c r="O63" s="10" t="n"/>
+      <c r="P63" s="10" t="n"/>
+      <c r="Q63" s="9" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q46"/>
+  <autoFilter ref="A1:Q63"/>
   <dataValidations count="4">
     <dataValidation sqref="E2:E245" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"P0,P1,P2"</formula1>
@@ -4106,7 +5317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4131,7 +5342,7 @@
         </is>
       </c>
       <c r="B3" s="15" t="n">
-        <v>45</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4">
@@ -4141,7 +5352,7 @@
         </is>
       </c>
       <c r="B4" s="15" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5">
@@ -4151,7 +5362,7 @@
         </is>
       </c>
       <c r="B5" s="15" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6">
@@ -4161,7 +5372,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7">
@@ -4171,7 +5382,7 @@
         </is>
       </c>
       <c r="B7" s="15" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8">
@@ -4302,7 +5513,7 @@
         </is>
       </c>
       <c r="B16" s="15" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C16" s="15" t="n">
         <v>2</v>
@@ -4312,7 +5523,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>覆盖快捷键状态、开机自启、目录打开、Markdown 导出。</t>
+          <t>覆盖快捷键状态、开机自启、目录打开、Markdown 导出及知识元数据。</t>
         </is>
       </c>
     </row>
@@ -4323,223 +5534,431 @@
         </is>
       </c>
       <c r="B17" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="C17" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="C17" s="15" t="n">
+      <c r="D17" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>覆盖托盘、退出前 flush、重启持久化及知识备份恢复。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>知识节点</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D17" s="15" t="n">
+      <c r="C18" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D18" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>覆盖沉淀、唯一标题、移出和历史标题。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>知识关联</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="C19" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D19" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 WikiLink 补全、出链/反链、未解析与刷新。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>增强搜索</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>覆盖托盘、退出前 flush、重启后的数据保留。</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="C20" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 trigram、排名片段、短查询回退和视图筛选。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>索引维护</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>覆盖搜索与关系索引的安全重建。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>建议每轮第二阶段提交至少执行的最小回归集</t>
         </is>
       </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="B24" s="4" t="n"/>
+      <c r="C24" s="4" t="n"/>
+      <c r="D24" s="4" t="n"/>
+      <c r="E24" s="5" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>用例ID</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>理由</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="15" t="inlineStr">
-        <is>
-          <t>QC-01</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>验证全局快捷键主入口</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="15" t="inlineStr">
-        <is>
-          <t>QC-06</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>验证草稿恢复链路</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="15" t="inlineStr">
-        <is>
-          <t>QC-07</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>验证快速记录提交到主列表</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="15" t="inlineStr">
-        <is>
-          <t>IN-01</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>验证收集箱默认过滤</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>IN-04</t>
+          <t>QC-01</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>验证详情自动保存</t>
+          <t>验证全局快捷键主入口</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>IN-05</t>
+          <t>QC-06</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>验证切换条目前 flush</t>
+          <t>验证草稿恢复链路</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>IN-07</t>
+          <t>QC-07</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>验证原始内容不被覆盖</t>
+          <t>验证快速记录提交到主列表</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>SF-06</t>
+          <t>IN-01</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>验证状态筛选与收集箱语义</t>
+          <t>验证收集箱默认过滤</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="15" t="inlineStr">
         <is>
-          <t>TR-01</t>
+          <t>IN-04</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>验证移到回收站</t>
+          <t>验证详情自动保存</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="15" t="inlineStr">
         <is>
-          <t>TR-02</t>
+          <t>IN-05</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>验证回收站恢复</t>
+          <t>验证切换条目前 flush</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="15" t="inlineStr">
         <is>
-          <t>EX-01</t>
+          <t>IN-07</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>验证导出总量与范围</t>
+          <t>验证原始内容不被覆盖</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="15" t="inlineStr">
         <is>
-          <t>DS-01</t>
+          <t>SF-06</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>验证主窗口关闭到托盘</t>
+          <t>验证状态筛选与收集箱语义</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="15" t="inlineStr">
         <is>
-          <t>DS-03</t>
+          <t>TR-01</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>验证退出前主窗口 flush</t>
+          <t>验证移到回收站</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="15" t="inlineStr">
         <is>
-          <t>DS-04</t>
+          <t>TR-02</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>验证退出前快速记录 flush</t>
+          <t>验证回收站恢复</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="15" t="inlineStr">
         <is>
+          <t>EX-01</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>验证导出总量与范围</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="15" t="inlineStr">
+        <is>
+          <t>DS-01</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>验证主窗口关闭到托盘</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="15" t="inlineStr">
+        <is>
+          <t>DS-03</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>验证退出前主窗口 flush</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="15" t="inlineStr">
+        <is>
+          <t>DS-04</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>验证退出前快速记录 flush</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="15" t="inlineStr">
+        <is>
           <t>DS-05</t>
         </is>
       </c>
-      <c r="B36" s="3" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>验证重启后的持久化</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="15" t="inlineStr">
+        <is>
+          <t>KB-01</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>验证沉淀与收集箱分离</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="15" t="inlineStr">
+        <is>
+          <t>KB-02</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>验证标题唯一性与不丢内容</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="15" t="inlineStr">
+        <is>
+          <t>KB-04</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>验证历史标题继续解析</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="15" t="inlineStr">
+        <is>
+          <t>LK-01</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>验证 WikiLink 补全</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="15" t="inlineStr">
+        <is>
+          <t>LK-02</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>验证出链、反链和 occurrence</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="15" t="inlineStr">
+        <is>
+          <t>LK-04</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>验证跨窗口反链刷新</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="15" t="inlineStr">
+        <is>
+          <t>SR-01</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>验证三字中文 trigram 搜索</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="15" t="inlineStr">
+        <is>
+          <t>SR-03</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>验证短查询 LIKE 回退</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="15" t="inlineStr">
+        <is>
+          <t>IX-01</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>验证重建索引不改用户数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="15" t="inlineStr">
+        <is>
+          <t>DS-06</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>验证备份恢复知识数据与反链</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A24:E24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>